<commit_message>
nearby search - ready for 1st test
</commit_message>
<xml_diff>
--- a/assets/Partner Launch - Airport List.xlsx
+++ b/assets/Partner Launch - Airport List.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\avtopia\data_sync_desktop\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbaszler\Source\repos\jaredbaszler\data_sync_desktop\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A99D3BB-AE50-439C-A6E3-2BBC1863B0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="July 1 Launch" sheetId="1" r:id="rId1"/>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="211">
   <si>
     <t>Van Nuys (VNY)</t>
   </si>
@@ -652,12 +651,24 @@
   </si>
   <si>
     <t>Google:NumReviews</t>
+  </si>
+  <si>
+    <t>Google:PriceLevel</t>
+  </si>
+  <si>
+    <t>Google:GlobalCode</t>
+  </si>
+  <si>
+    <t>Google:CompoundCode</t>
+  </si>
+  <si>
+    <t>Google:OpeningHours</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -757,7 +768,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -780,7 +791,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1094,16 +1104,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B78"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.7109375" style="2"/>
+    <col min="1" max="1" width="48.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>35</v>
       </c>
@@ -1111,7 +1121,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1119,7 +1129,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -1127,7 +1137,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -1135,7 +1145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>43</v>
       </c>
@@ -1143,7 +1153,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -1151,7 +1161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>41</v>
       </c>
@@ -1159,7 +1169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>42</v>
       </c>
@@ -1167,7 +1177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
@@ -1183,7 +1193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1191,7 +1201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
@@ -1199,7 +1209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>22</v>
       </c>
@@ -1207,7 +1217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -1215,7 +1225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>38</v>
       </c>
@@ -1223,7 +1233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>40</v>
       </c>
@@ -1231,7 +1241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>39</v>
       </c>
@@ -1239,7 +1249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>44</v>
       </c>
@@ -1247,7 +1257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>46</v>
       </c>
@@ -1255,7 +1265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>45</v>
       </c>
@@ -1263,7 +1273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>47</v>
       </c>
@@ -1271,7 +1281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>48</v>
       </c>
@@ -1279,7 +1289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>49</v>
       </c>
@@ -1287,7 +1297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>50</v>
       </c>
@@ -1295,7 +1305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>51</v>
       </c>
@@ -1303,7 +1313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>52</v>
       </c>
@@ -1311,7 +1321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>53</v>
       </c>
@@ -1319,7 +1329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>54</v>
       </c>
@@ -1327,7 +1337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>55</v>
       </c>
@@ -1335,7 +1345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>90</v>
       </c>
@@ -1343,7 +1353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>15</v>
       </c>
@@ -1351,7 +1361,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>57</v>
       </c>
@@ -1359,7 +1369,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>58</v>
       </c>
@@ -1367,7 +1377,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>59</v>
       </c>
@@ -1375,7 +1385,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>60</v>
       </c>
@@ -1383,7 +1393,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1391,7 +1401,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>56</v>
       </c>
@@ -1399,7 +1409,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>2</v>
       </c>
@@ -1407,7 +1417,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
@@ -1415,7 +1425,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>14</v>
       </c>
@@ -1423,7 +1433,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>32</v>
       </c>
@@ -1431,7 +1441,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>34</v>
       </c>
@@ -1439,7 +1449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>83</v>
       </c>
@@ -1447,7 +1457,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>84</v>
       </c>
@@ -1455,7 +1465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>85</v>
       </c>
@@ -1463,7 +1473,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>86</v>
       </c>
@@ -1471,7 +1481,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>87</v>
       </c>
@@ -1479,7 +1489,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>88</v>
       </c>
@@ -1487,7 +1497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>89</v>
       </c>
@@ -1495,7 +1505,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>20</v>
       </c>
@@ -1503,7 +1513,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>91</v>
       </c>
@@ -1511,7 +1521,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>67</v>
       </c>
@@ -1519,7 +1529,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>69</v>
       </c>
@@ -1527,7 +1537,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>27</v>
       </c>
@@ -1535,7 +1545,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>25</v>
       </c>
@@ -1543,7 +1553,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>62</v>
       </c>
@@ -1551,7 +1561,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>63</v>
       </c>
@@ -1559,7 +1569,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>64</v>
       </c>
@@ -1567,7 +1577,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>18</v>
       </c>
@@ -1575,7 +1585,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>23</v>
       </c>
@@ -1583,7 +1593,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>65</v>
       </c>
@@ -1591,7 +1601,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>7</v>
       </c>
@@ -1599,7 +1609,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>66</v>
       </c>
@@ -1607,7 +1617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>79</v>
       </c>
@@ -1615,7 +1625,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>82</v>
       </c>
@@ -1623,7 +1633,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>31</v>
       </c>
@@ -1631,7 +1641,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>33</v>
       </c>
@@ -1639,7 +1649,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>71</v>
       </c>
@@ -1647,7 +1657,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>70</v>
       </c>
@@ -1655,7 +1665,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>72</v>
       </c>
@@ -1663,7 +1673,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>73</v>
       </c>
@@ -1671,7 +1681,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>74</v>
       </c>
@@ -1679,7 +1689,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>75</v>
       </c>
@@ -1687,7 +1697,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>76</v>
       </c>
@@ -1695,7 +1705,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>77</v>
       </c>
@@ -1703,7 +1713,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>81</v>
       </c>
@@ -1711,7 +1721,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>12</v>
       </c>
@@ -1719,7 +1729,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>78</v>
       </c>
@@ -1728,8 +1738,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B78" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B78">
+  <autoFilter ref="A1:B78"/>
+  <sortState ref="A2:B78">
     <sortCondition ref="B2:B78"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1738,20 +1748,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:E33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.28515625" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.33203125" customWidth="1"/>
+    <col min="4" max="4" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>35</v>
       </c>
@@ -1768,7 +1778,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>92</v>
       </c>
@@ -1785,7 +1795,7 @@
         <v>-111.91100311279</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>93</v>
       </c>
@@ -1802,7 +1812,7 @@
         <v>-112.012001037597</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>94</v>
       </c>
@@ -1819,7 +1829,7 @@
         <v>-118.48999786377</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>95</v>
       </c>
@@ -1836,7 +1846,7 @@
         <v>-118.15200040000001</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>96</v>
       </c>
@@ -1853,7 +1863,7 @@
         <v>-117.86799619999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -1870,7 +1880,7 @@
         <v>-39.253101000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>98</v>
       </c>
@@ -1887,7 +1897,7 @@
         <v>-122.221001</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>99</v>
       </c>
@@ -1904,7 +1914,7 @@
         <v>48.516666412353501</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>100</v>
       </c>
@@ -1921,7 +1931,7 @@
         <v>-118.450996</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>101</v>
       </c>
@@ -1938,7 +1948,7 @@
         <v>-121.929001</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>102</v>
       </c>
@@ -1955,7 +1965,7 @@
         <v>-118.359001159667</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>103</v>
       </c>
@@ -1972,7 +1982,7 @@
         <v>-119.8399963</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -1989,7 +1999,7 @@
         <v>-116.98000335693</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>105</v>
       </c>
@@ -2006,7 +2016,7 @@
         <v>-104.84899900000001</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>106</v>
       </c>
@@ -2023,7 +2033,7 @@
         <v>-106.8690033</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>107</v>
       </c>
@@ -2040,7 +2050,7 @@
         <v>-80.095596313476506</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -2057,7 +2067,7 @@
         <v>-80.278396999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>109</v>
       </c>
@@ -2074,7 +2084,7 @@
         <v>-80.152702000000005</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>110</v>
       </c>
@@ -2091,7 +2101,7 @@
         <v>-81.332901000000007</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>111</v>
       </c>
@@ -2108,7 +2118,7 @@
         <v>-80.107696533199999</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>112</v>
       </c>
@@ -2125,7 +2135,7 @@
         <v>-81.437103271500007</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>113</v>
       </c>
@@ -2142,7 +2152,7 @@
         <v>-84.302001953100003</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>114</v>
       </c>
@@ -2159,7 +2169,7 @@
         <v>-97.433098000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>115</v>
       </c>
@@ -2176,7 +2186,7 @@
         <v>-97.652198791503906</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>116</v>
       </c>
@@ -2193,7 +2203,7 @@
         <v>-71.289001459999994</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>117</v>
       </c>
@@ -2210,7 +2220,7 @@
         <v>-74.060798645000006</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>118</v>
       </c>
@@ -2227,7 +2237,7 @@
         <v>-74.414901733398395</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>119</v>
       </c>
@@ -2244,7 +2254,7 @@
         <v>-73.707603454589801</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>120</v>
       </c>
@@ -2261,7 +2271,7 @@
         <v>-96.851799</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>121</v>
       </c>
@@ -2278,7 +2288,7 @@
         <v>-95.278900149999998</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>122</v>
       </c>
@@ -2295,7 +2305,7 @@
         <v>-97.038002000000006</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>123</v>
       </c>
@@ -2313,60 +2323,60 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:C1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AV1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AZ1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="24.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="32" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="15" max="19" width="14" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="11" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="19" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="17" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="19.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:52" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>159</v>
       </c>
@@ -2445,74 +2455,87 @@
       <c r="Z1" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="AA1" s="14" t="s">
+      <c r="AA1" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="AB1" s="14" t="s">
+      <c r="AB1" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="AC1" s="14" t="s">
+      <c r="AC1" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="AD1" s="14" t="s">
+      <c r="AD1" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="AE1" s="14" t="s">
+      <c r="AE1" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="AF1" s="14" t="s">
+      <c r="AF1" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="AG1" s="14" t="s">
+      <c r="AG1" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="AH1" s="14" t="s">
+      <c r="AH1" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="AI1" s="14" t="s">
+      <c r="AI1" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="AJ1" s="14" t="s">
+      <c r="AJ1" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="AK1" s="14" t="s">
+      <c r="AK1" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="AL1" s="14" t="s">
+      <c r="AL1" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="AM1" s="14" t="s">
+      <c r="AM1" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="AN1" s="14" t="s">
+      <c r="AN1" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="AO1" s="14" t="s">
+      <c r="AO1" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="AP1" s="14" t="s">
+      <c r="AP1" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="AQ1" s="14" t="s">
+      <c r="AQ1" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="AR1" s="14" t="s">
+      <c r="AR1" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="AS1" s="14" t="s">
+      <c r="AS1" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="AT1" s="14" t="s">
+      <c r="AT1" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="AU1" s="14" t="s">
+      <c r="AU1" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="AV1" s="14" t="s">
+      <c r="AV1" s="10" t="s">
         <v>206</v>
+      </c>
+      <c r="AW1" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="AX1" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="AY1" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="AZ1" s="10" t="s">
+        <v>210</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>